<commit_message>
[ Data ] Update localized content tables
</commit_message>
<xml_diff>
--- a/Assets/RawData/Excel/Text/TextTableData.xlsx
+++ b/Assets/RawData/Excel/Text/TextTableData.xlsx
@@ -3,81 +3,483 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\TinyHero\Assets\RawData\Excel\Text\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CA6544B-0916-44E2-94A6-9ECD9445C447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="TextTableData" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <fileRecoveryPr autoRecover="0" crashSave="0" dataExtractLoad="0" repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
-  <si>
-    <t>TextKey</t>
-  </si>
-  <si>
-    <t>KR</t>
-  </si>
-  <si>
-    <t>EN</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_COMMON_CONFIRM</t>
-  </si>
-  <si>
-    <t>확인</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_COMMON_CANCEL</t>
-  </si>
-  <si>
-    <t>취소</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_COMMON_CLOSE</t>
-  </si>
-  <si>
-    <t>닫기</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_SAVE_COMPLETE</t>
-  </si>
-  <si>
-    <t>저장이 완료되었습니다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_SAVE_FAILED</t>
-  </si>
-  <si>
-    <t>저장에 실패했습니다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_MAP_LOADING_DATA</t>
-  </si>
-  <si>
-    <t>맵 데이터를 불러오는 중...</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_MAP_LOADING_COMPLETE</t>
-  </si>
-  <si>
-    <t>로딩 완료</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="144">
+  <si>
+    <t xml:space="preserve">TextKey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_COMMON_CONFIRM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">확인</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_COMMON_CANCEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">취소</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_COMMON_CLOSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">닫기</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_SAVE_COMPLETE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저장이 완료되었습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_SAVE_FAILED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저장에 실패했습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_MAP_LOADING_DATA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">맵 데이터를 불러오는 중...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_MAP_LOADING_COMPLETE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">로딩 완료</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CONSUMABLE_CUBE_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미스틱 큐브</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CONSUMABLE_CUBE_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">신비한 힘이 깃든 큐브.
+아이템의 잠재능력을 일깨워준다고 알려져 있다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CONSUMABLE_SKILLBOOK_SHADOW_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">섀도우 파트너 스킬북</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CONSUMABLE_SKILLBOOK_SHADOW_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">섀도우 파트너를 배울 수 있는 스킬북이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CURRENCY_GOLD_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">골드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CURRENCY_GOLD_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">반짝거리는 재화이다.
+어딜가든 공용재화로 취급된다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_BRONZE_SWORD_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">브론즈 소드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_BRONZE_SWORD_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">여기저기서 흔하게 볼 수 있는 검이다.
+대충 쓸만해보인다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_ANGEL_KNIG_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엔젤나이트 헬멧</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_ANGEL_KNIG_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">천상의 기사단장이 착용했다고 알려진 장비 중 하나.
+보고 있기만 해도 신성한 힘이 느껴지는 듯 하다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_DREX_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">드렉스의 투구</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_DREX_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">드렉스가 항상 착용 중인 투구이다.
+똑같이 생긴 투구가 여러개 있음이 틀림없다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_GOLD_KNIGH_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">골드나이트 헬멧</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_GOLD_KNIGH_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">금빛으로 빛나는 기사의 투구이다.
+해가 비추면 눈이 너무 아픈 것 같기도..?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_ANGEL_KNIGH_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엔젤나이트 소드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_ANGEL_KNIGH_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_GOLD_KNIGHT_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">골드나이트 소드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_GOLD_KNIGHT_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">금빛으로 빛나는 기사의 검이다.
+해가 비추면 눈이 너무 아픈 것 같기도..?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_IGNITION_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이그니션 소드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_IGNITION_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">불꽃의 힘이 깃든 검이다.
+주위에 두기만 해도 뜨거운 열기가 느껴진다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_MATERIAL_HONEY_JELLY_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">허니젤리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_MATERIAL_HONEY_JELLY_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">달콤한 향이 나는 허니 젤리다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_MATERIAL_TURTLE_SNAIL_WATER_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거북 달팽이의 점액</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_MATERIAL_TURTLE_SNAIL_WATER_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">끈적끈적한 점액이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_QUEST_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잊지 못한 향기</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">드렉스에게 고민이 있는 것일까?
+무슨 일인지 물어보자.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">분명 하나 쯤은 떨어져 있을텐데...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">오, 자네인가?
+마침 잘 왔네.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">최근에 무슨 금색 젤리같은 것을 먹었는데
+너무 맛있어서 잊을 수가 없다네.
+향도 아주 좋았지.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">근처 몬스터를 잡으면 나온다던데,
+몇 개만 가져다 줄 수 있겠나?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_01_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">호오 그래, 이 향기야.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_02_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">정말 고맙네.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_03_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">좋은 하루 보내게.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_QUEST_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그라함의 고민</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그의 얼굴엔 근심이 가득하다.
+무슨 일인지 물어볼까?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잡아도 잡아도 끝이 없군..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">오, 그래 자네인가?
+혹시 마을을 위해 부탁을 좀 들어줄 수 있겠나?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">요새 마을 주변에 돌아다니는 몬스터 때문일세.
+잡아도 잡아도 끝이 없다네..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그 놈들 좀 처치해주게.
+자네만 믿겠네.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_02_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_03_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이젠 그 놈들 수가 좀 줄었겠지..
+자네는 역시 믿고 맡길 수 있어서 좋군.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_QUEST_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">성장을 위한 첫 걸음</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">촌장에게 성장을 위한 가르침을 받자.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그래, 자네인가?
+무슨 일인가?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">성장이라..
+오랜만에 자네와 같은 열정적인 눈빛을 보는군..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">좋네.
+먼저, 이 앞 숲으로 가서 몬스터를 몇 마리 처치한 후, 전리품을 가져오게.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">성장엔 실전경험이 가장 중요한 법.
+갔다오게.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_01_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">왔는가?
+수고했네.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_02_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">어떤가, 실제로 몬스터를 상대한다는 건 만만치 않았을테지.
+훈련용 밀짚인형으로 연습하던 것과는 또 다른 느낌이였을게야.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_03_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">앞으로 정진하게.
+연습과 실전만이 자네를 더 높은 곳으로 성장시켜줄테니.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_ARC_BOLT_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">아크볼트</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_ARC_BOLT_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">번개의 힘이 깃든 에너지 볼을 전방으로 발사한다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_BLIZARD_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">블리자드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_BLIZARD_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">하늘길을 열어 얼음 결정을 수엎이 쏟아붇는다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_DOUBLE_JUMP_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">더블 점프</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_DOUBLE_JUMP_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">신성한 힘을 응축 시킨 후, 점프 후 공중에서 한 번 더 도약한다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_FLAME_SLASH_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">플레임 슬래시</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_FLAME_SLASH_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">검날에 불꽃을 입혀 전방에 휘두른다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_MOON_BLADE_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">문 블레이드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_MOON_BLADE_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">달빛의 힘을 실은 검기를 전방으로 날린다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_SHADOW_PARTNER_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">섀도우 파트너</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_SHADOW_PARTNER_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">어둠의 힘을 그림자에 깃들게한다.
+나의 행동을 복제하는 그림자 분신을 생성한다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_WIND_DANCE_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">윈드 댄스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_WIND_DANCE_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바람 속에 녹아들어 시야에 들어온 모든 적들을 번갈아 가며 타격한다.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -129,11 +531,11 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -350,6 +752,7 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
@@ -357,6 +760,7 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
@@ -364,6 +768,7 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
           <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
@@ -427,7 +832,7 @@
   <a:objectDefaults>
     <a:lnDef>
       <a:spPr/>
-      <a:bodyPr/>
+      <a:bodyPr rtlCol="0"/>
       <a:lstStyle/>
       <a:style>
         <a:lnRef idx="2">
@@ -455,8 +860,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="36" customWidth="1"/>
@@ -550,6 +955,710 @@
         <v>15</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" t="s">
+        <v>64</v>
+      </c>
+      <c r="C32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>69</v>
+      </c>
+      <c r="B35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B37" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>75</v>
+      </c>
+      <c r="B38" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" t="s">
+        <v>78</v>
+      </c>
+      <c r="C39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>79</v>
+      </c>
+      <c r="B40" t="s">
+        <v>80</v>
+      </c>
+      <c r="C40" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>81</v>
+      </c>
+      <c r="B41" t="s">
+        <v>82</v>
+      </c>
+      <c r="C41" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>83</v>
+      </c>
+      <c r="B42" t="s">
+        <v>84</v>
+      </c>
+      <c r="C42" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>85</v>
+      </c>
+      <c r="B43" t="s">
+        <v>86</v>
+      </c>
+      <c r="C43" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>87</v>
+      </c>
+      <c r="B44" t="s">
+        <v>88</v>
+      </c>
+      <c r="C44" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>89</v>
+      </c>
+      <c r="B45" t="s">
+        <v>90</v>
+      </c>
+      <c r="C45" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>91</v>
+      </c>
+      <c r="B46" t="s">
+        <v>92</v>
+      </c>
+      <c r="C46" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>93</v>
+      </c>
+      <c r="B47" t="s">
+        <v>94</v>
+      </c>
+      <c r="C47" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>95</v>
+      </c>
+      <c r="B48" t="s">
+        <v>80</v>
+      </c>
+      <c r="C48" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" t="s">
+        <v>97</v>
+      </c>
+      <c r="C49" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>100</v>
+      </c>
+      <c r="B51" t="s">
+        <v>101</v>
+      </c>
+      <c r="C51" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" t="s">
+        <v>103</v>
+      </c>
+      <c r="C52" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" t="s">
+        <v>105</v>
+      </c>
+      <c r="C53" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>106</v>
+      </c>
+      <c r="B54" t="s">
+        <v>107</v>
+      </c>
+      <c r="C54" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>108</v>
+      </c>
+      <c r="B55" t="s">
+        <v>109</v>
+      </c>
+      <c r="C55" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>110</v>
+      </c>
+      <c r="B56" t="s">
+        <v>111</v>
+      </c>
+      <c r="C56" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>112</v>
+      </c>
+      <c r="B57" t="s">
+        <v>113</v>
+      </c>
+      <c r="C57" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>114</v>
+      </c>
+      <c r="B58" t="s">
+        <v>115</v>
+      </c>
+      <c r="C58" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>116</v>
+      </c>
+      <c r="B59" t="s">
+        <v>117</v>
+      </c>
+      <c r="C59" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>118</v>
+      </c>
+      <c r="B60" t="s">
+        <v>119</v>
+      </c>
+      <c r="C60" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>120</v>
+      </c>
+      <c r="B61" t="s">
+        <v>121</v>
+      </c>
+      <c r="C61" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>122</v>
+      </c>
+      <c r="B62" t="s">
+        <v>123</v>
+      </c>
+      <c r="C62" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>124</v>
+      </c>
+      <c r="B63" t="s">
+        <v>125</v>
+      </c>
+      <c r="C63" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>126</v>
+      </c>
+      <c r="B64" t="s">
+        <v>127</v>
+      </c>
+      <c r="C64" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>128</v>
+      </c>
+      <c r="B65" t="s">
+        <v>129</v>
+      </c>
+      <c r="C65" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>130</v>
+      </c>
+      <c r="B66" t="s">
+        <v>131</v>
+      </c>
+      <c r="C66" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>132</v>
+      </c>
+      <c r="B67" t="s">
+        <v>133</v>
+      </c>
+      <c r="C67" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>134</v>
+      </c>
+      <c r="B68" t="s">
+        <v>135</v>
+      </c>
+      <c r="C68" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>136</v>
+      </c>
+      <c r="B69" t="s">
+        <v>137</v>
+      </c>
+      <c r="C69" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>138</v>
+      </c>
+      <c r="B70" t="s">
+        <v>139</v>
+      </c>
+      <c r="C70" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>140</v>
+      </c>
+      <c r="B71" t="s">
+        <v>141</v>
+      </c>
+      <c r="C71" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>142</v>
+      </c>
+      <c r="B72" t="s">
+        <v>143</v>
+      </c>
+      <c r="C72" t="s">
+        <v>142</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
[ Data ] Update text table test content
</commit_message>
<xml_diff>
--- a/Assets/RawData/Excel/Text/TextTableData.xlsx
+++ b/Assets/RawData/Excel/Text/TextTableData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\TinyHero\Assets\RawData\Excel\Text\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9E829AE-8D95-4634-9C2F-CF8264D487B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB02C98-32F9-446C-9351-9BDABBC2C91D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38805" yWindow="0" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="0" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TextTableData" sheetId="1" r:id="rId1"/>
@@ -115,9 +115,6 @@
     <t>KEY_TEXT_ITEM_EQUIPMENT_BRONZE_SWORD_ITEM_NAME</t>
   </si>
   <si>
-    <t>브론즈 소드</t>
-  </si>
-  <si>
     <t>KEY_TEXT_ITEM_EQUIPMENT_BRONZE_SWORD_DESCRIPTION</t>
   </si>
   <si>
@@ -206,9 +203,6 @@
   </si>
   <si>
     <t>KEY_TEXT_ITEM_MATERIAL_HONEY_JELLY_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>달콤한 향이 나는 허니 젤리다.</t>
   </si>
   <si>
     <t>KEY_TEXT_ITEM_MATERIAL_TURTLE_SNAIL_WATER_ITEM_NAME</t>
@@ -722,6 +716,123 @@
         <family val="2"/>
       </rPr>
       <t>?</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>달콤한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>향이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>나는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>허니</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>젤리다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>초보자의 브론즈</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>소드</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -786,13 +897,16 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1288,12 +1402,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" ht="16.5">
       <c r="A15" t="s">
         <v>29</v>
       </c>
-      <c r="B15" t="s">
-        <v>30</v>
+      <c r="B15" s="3" t="s">
+        <v>184</v>
       </c>
       <c r="C15" t="s">
         <v>29</v>
@@ -1301,860 +1415,860 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
         <v>31</v>
       </c>
-      <c r="B16" t="s">
-        <v>32</v>
-      </c>
       <c r="C16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
         <v>33</v>
       </c>
-      <c r="B17" t="s">
-        <v>34</v>
-      </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" t="s">
         <v>35</v>
       </c>
-      <c r="B18" t="s">
-        <v>36</v>
-      </c>
       <c r="C18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
         <v>37</v>
       </c>
-      <c r="B19" t="s">
-        <v>38</v>
-      </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" t="s">
         <v>39</v>
       </c>
-      <c r="B20" t="s">
-        <v>40</v>
-      </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
         <v>41</v>
       </c>
-      <c r="B21" t="s">
-        <v>42</v>
-      </c>
       <c r="C21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
         <v>43</v>
       </c>
-      <c r="B22" t="s">
-        <v>44</v>
-      </c>
       <c r="C22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" t="s">
         <v>45</v>
       </c>
-      <c r="B23" t="s">
-        <v>46</v>
-      </c>
       <c r="C23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" t="s">
         <v>48</v>
       </c>
-      <c r="B25" t="s">
-        <v>49</v>
-      </c>
       <c r="C25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" t="s">
         <v>50</v>
       </c>
-      <c r="B26" t="s">
-        <v>51</v>
-      </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" t="s">
         <v>52</v>
       </c>
-      <c r="B27" t="s">
-        <v>53</v>
-      </c>
       <c r="C27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" t="s">
         <v>54</v>
       </c>
-      <c r="B28" t="s">
-        <v>55</v>
-      </c>
       <c r="C28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" t="s">
         <v>56</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="16.5">
+      <c r="A30" t="s">
         <v>57</v>
       </c>
-      <c r="C29" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>58</v>
-      </c>
-      <c r="B30" t="s">
-        <v>59</v>
+      <c r="B30" s="3" t="s">
+        <v>183</v>
       </c>
       <c r="C30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B31" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C31" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B32" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C32" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B33" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C33" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B34" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C34" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B35" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B36" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B38" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C38" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B39" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C39" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C40" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B41" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C41" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B42" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C42" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B43" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C43" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B44" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C44" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B45" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C45" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B46" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C46" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B47" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C47" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B48" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C48" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B49" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C49" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B50" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C50" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B51" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C51" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B52" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C52" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B53" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C53" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B54" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C54" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B55" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C55" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B56" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C56" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B57" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C57" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B58" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C58" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B59" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C59" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B60" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C60" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B61" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C61" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B62" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C62" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B63" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C63" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B64" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C64" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B65" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C65" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B66" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C66" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B67" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C67" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B68" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C68" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B69" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C69" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B70" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C70" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B71" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C71" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B72" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C72" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B73" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C73" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B74" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C74" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B75" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C75" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B76" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C76" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B77" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C77" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B78" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C78" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B79" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C79" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B80" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C80" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="14.25" customHeight="1">
       <c r="A81" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C81" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B82" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C82" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B83" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C83" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B84" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C84" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B85" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C85" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B86" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C86" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B87" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C87" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B88" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C88" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B89" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C89" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B90" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C90" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B91" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C91" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B92" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C92" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B93" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C93" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[ UI ] Improve content download completion flow
</commit_message>
<xml_diff>
--- a/Assets/RawData/Excel/Text/TextTableData.xlsx
+++ b/Assets/RawData/Excel/Text/TextTableData.xlsx
@@ -3,598 +3,592 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\TinyHero\Assets\RawData\Excel\Text\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB02C98-32F9-446C-9351-9BDABBC2C91D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="0" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="0" windowWidth="28800" windowHeight="15345"/>
   </bookViews>
   <sheets>
     <sheet name="TextTableData" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr autoRecover="0"/>
+  <fileRecoveryPr autoRecover="0" crashSave="0" dataExtractLoad="0" repairLoad="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="185">
-  <si>
-    <t>TextKey</t>
-  </si>
-  <si>
-    <t>KR</t>
-  </si>
-  <si>
-    <t>EN</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_COMMON_CONFIRM</t>
-  </si>
-  <si>
-    <t>확인</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_COMMON_CANCEL</t>
-  </si>
-  <si>
-    <t>취소</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_COMMON_CLOSE</t>
-  </si>
-  <si>
-    <t>닫기</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_SAVE_COMPLETE</t>
-  </si>
-  <si>
-    <t>저장이 완료되었습니다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_UI_SAVE_FAILED</t>
-  </si>
-  <si>
-    <t>저장에 실패했습니다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_MAP_LOADING_DATA</t>
-  </si>
-  <si>
-    <t>맵 데이터를 불러오는 중...</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_MAP_LOADING_COMPLETE</t>
-  </si>
-  <si>
-    <t>로딩 완료</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_CONSUMABLE_CUBE_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>미스틱 큐브</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_CONSUMABLE_CUBE_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>신비한 힘이 깃든 큐브.
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="195">
+  <si>
+    <t xml:space="preserve">TextKey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_COMMON_CONFIRM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">확인</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_COMMON_CANCEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">취소</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_COMMON_CLOSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">닫기</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_SAVE_COMPLETE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저장이 완료되었습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_SAVE_FAILED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">저장에 실패했습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_MAP_LOADING_DATA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">맵 데이터를 불러오는 중...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_MAP_LOADING_COMPLETE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">로딩 완료</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CONSUMABLE_CUBE_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미스틱 큐브</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CONSUMABLE_CUBE_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">신비한 힘이 깃든 큐브.
 아이템의 잠재능력을 일깨워준다고 알려져 있다.</t>
   </si>
   <si>
-    <t>KEY_TEXT_ITEM_CONSUMABLE_SKILLBOOK_SHADOW_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>섀도우 파트너 스킬북</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_CONSUMABLE_SKILLBOOK_SHADOW_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>섀도우 파트너를 배울 수 있는 스킬북이다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_CURRENCY_GOLD_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>골드</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_CURRENCY_GOLD_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>반짝거리는 재화이다.
+    <t xml:space="preserve">KEY_TEXT_ITEM_CONSUMABLE_SKILLBOOK_SHADOW_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">섀도우 파트너 스킬북</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CONSUMABLE_SKILLBOOK_SHADOW_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">섀도우 파트너를 배울 수 있는 스킬북이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CURRENCY_GOLD_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">골드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_CURRENCY_GOLD_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">반짝거리는 재화이다.
 어딜가든 공용재화로 취급된다.</t>
   </si>
   <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_BRONZE_SWORD_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_BRONZE_SWORD_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>여기저기서 흔하게 볼 수 있는 검이다.
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_BRONZE_SWORD_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_BRONZE_SWORD_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">여기저기서 흔하게 볼 수 있는 검이다.
 대충 쓸만해보인다.</t>
   </si>
   <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_HELMET_ANGEL_KNIG_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>엔젤나이트 헬멧</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_HELMET_ANGEL_KNIG_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>천상의 기사단장이 착용했다고 알려진 장비 중 하나.
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_ANGEL_KNIG_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엔젤나이트 헬멧</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_ANGEL_KNIG_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">천상의 기사단장이 착용했다고 알려진 장비 중 하나.
 보고 있기만 해도 신성한 힘이 느껴지는 듯 하다.</t>
   </si>
   <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_HELMET_DREX_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>드렉스의 투구</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_HELMET_DREX_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>드렉스가 항상 착용 중인 투구이다.
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_DREX_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">드렉스의 투구</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_DREX_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">드렉스가 항상 착용 중인 투구이다.
 똑같이 생긴 투구가 여러개 있음이 틀림없다.</t>
   </si>
   <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_HELMET_GOLD_KNIGH_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>골드나이트 헬멧</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_HELMET_GOLD_KNIGH_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>금빛으로 빛나는 기사의 투구이다.
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_GOLD_KNIGH_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">골드나이트 헬멧</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_HELMET_GOLD_KNIGH_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">금빛으로 빛나는 기사의 투구이다.
 해가 비추면 눈이 너무 아픈 것 같기도..?</t>
   </si>
   <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_SWORD_ANGEL_KNIGH_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>엔젤나이트 소드</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_SWORD_ANGEL_KNIGH_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_SWORD_GOLD_KNIGHT_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>골드나이트 소드</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_SWORD_GOLD_KNIGHT_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>금빛으로 빛나는 기사의 검이다.
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_ANGEL_KNIGH_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엔젤나이트 소드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_ANGEL_KNIGH_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_GOLD_KNIGHT_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">골드나이트 소드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_GOLD_KNIGHT_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">금빛으로 빛나는 기사의 검이다.
 해가 비추면 눈이 너무 아픈 것 같기도..?</t>
   </si>
   <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_SWORD_IGNITION_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>이그니션 소드</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_EQUIPMENT_SWORD_IGNITION_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>불꽃의 힘이 깃든 검이다.
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_IGNITION_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이그니션 소드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_EQUIPMENT_SWORD_IGNITION_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">불꽃의 힘이 깃든 검이다.
 주위에 두기만 해도 뜨거운 열기가 느껴진다.</t>
   </si>
   <si>
-    <t>KEY_TEXT_ITEM_MATERIAL_HONEY_JELLY_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>허니젤리</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_MATERIAL_HONEY_JELLY_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_MATERIAL_TURTLE_SNAIL_WATER_ITEM_NAME</t>
-  </si>
-  <si>
-    <t>거북 달팽이의 점액</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_ITEM_MATERIAL_TURTLE_SNAIL_WATER_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>끈적끈적한 점액이다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_DREX_001_QUEST_NAME</t>
-  </si>
-  <si>
-    <t>잊지 못한 향기</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_DREX_001_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>드렉스에게 고민이 있는 것일까?
+    <t xml:space="preserve">KEY_TEXT_ITEM_MATERIAL_HONEY_JELLY_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">허니젤리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_MATERIAL_HONEY_JELLY_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_MATERIAL_TURTLE_SNAIL_WATER_ITEM_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거북 달팽이의 점액</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_ITEM_MATERIAL_TURTLE_SNAIL_WATER_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">끈적끈적한 점액이다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_QUEST_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잊지 못한 향기</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">드렉스에게 고민이 있는 것일까?
 무슨 일인지 물어보자.</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_01</t>
-  </si>
-  <si>
-    <t>분명 하나 쯤은 떨어져 있을텐데...</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_02</t>
-  </si>
-  <si>
-    <t>오, 자네인가?
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">분명 하나 쯤은 떨어져 있을텐데...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">오, 자네인가?
 마침 잘 왔네.</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_03</t>
-  </si>
-  <si>
-    <t>최근에 무슨 금색 젤리같은 것을 먹었는데
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">최근에 무슨 금색 젤리같은 것을 먹었는데
 너무 맛있어서 잊을 수가 없다네.
 향도 아주 좋았지.</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_04</t>
-  </si>
-  <si>
-    <t>근처 몬스터를 잡으면 나온다던데,
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">근처 몬스터를 잡으면 나온다던데,
 몇 개만 가져다 줄 수 있겠나?</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_01_02</t>
-  </si>
-  <si>
-    <t>호오 그래, 이 향기야.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_02_02</t>
-  </si>
-  <si>
-    <t>정말 고맙네.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_03_02</t>
-  </si>
-  <si>
-    <t>좋은 하루 보내게.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_001_QUEST_NAME</t>
-  </si>
-  <si>
-    <t>그라함의 고민</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_001_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>그의 얼굴엔 근심이 가득하다.
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_01_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">호오 그래, 이 향기야.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_02_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">정말 고맙네.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_DREX_001_DIALOGUE_LINE_LIST_03_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">좋은 하루 보내게.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_QUEST_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그라함의 고민</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그의 얼굴엔 근심이 가득하다.
 무슨 일인지 물어볼까?</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_01</t>
-  </si>
-  <si>
-    <t>잡아도 잡아도 끝이 없군..</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_02</t>
-  </si>
-  <si>
-    <t>오, 그래 자네인가?
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잡아도 잡아도 끝이 없군..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">오, 그래 자네인가?
 혹시 마을을 위해 부탁을 좀 들어줄 수 있겠나?</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_03</t>
-  </si>
-  <si>
-    <t>요새 마을 주변에 돌아다니는 몬스터 때문일세.
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">요새 마을 주변에 돌아다니는 몬스터 때문일세.
 잡아도 잡아도 끝이 없다네..</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_04</t>
-  </si>
-  <si>
-    <t>그 놈들 좀 처치해주게.
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그 놈들 좀 처치해주게.
 자네만 믿겠네.</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_02_02</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_03_02</t>
-  </si>
-  <si>
-    <t>이젠 그 놈들 수가 좀 줄었겠지..
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_02_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_001_DIALOGUE_LINE_LIST_03_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이젠 그 놈들 수가 좀 줄었겠지..
 자네는 역시 믿고 맡길 수 있어서 좋군.</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_002_QUEST_NAME</t>
-  </si>
-  <si>
-    <t>성장을 위한 첫 걸음</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_002_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>촌장에게 성장을 위한 가르침을 받자.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_01</t>
-  </si>
-  <si>
-    <t>그래, 자네인가?
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_QUEST_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">성장을 위한 첫 걸음</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">촌장에게 성장을 위한 가르침을 받자.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그래, 자네인가?
 무슨 일인가?</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_02</t>
-  </si>
-  <si>
-    <t>성장이라..
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">성장이라..
 오랜만에 자네와 같은 열정적인 눈빛을 보는군..</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_03</t>
-  </si>
-  <si>
-    <t>좋네.
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">좋네.
 먼저, 이 앞 숲으로 가서 몬스터를 몇 마리 처치한 후, 전리품을 가져오게.</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_04</t>
-  </si>
-  <si>
-    <t>성장엔 실전경험이 가장 중요한 법.
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">성장엔 실전경험이 가장 중요한 법.
 갔다오게.</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_01_02</t>
-  </si>
-  <si>
-    <t>왔는가?
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_01_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">왔는가?
 수고했네.</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_02_02</t>
-  </si>
-  <si>
-    <t>어떤가, 실제로 몬스터를 상대한다는 건 만만치 않았을테지.
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_02_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">어떤가, 실제로 몬스터를 상대한다는 건 만만치 않았을테지.
 훈련용 밀짚인형으로 연습하던 것과는 또 다른 느낌이였을게야.</t>
   </si>
   <si>
-    <t>KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_03_02</t>
-  </si>
-  <si>
-    <t>앞으로 정진하게.
+    <t xml:space="preserve">KEY_TEXT_QUEST_GRAHAM_002_DIALOGUE_LINE_LIST_03_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">앞으로 정진하게.
 연습과 실전만이 자네를 더 높은 곳으로 성장시켜줄테니.</t>
   </si>
   <si>
-    <t>KEY_TEXT_SKILL_ARC_BOLT_SKILL_NAME</t>
-  </si>
-  <si>
-    <t>아크볼트</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_ARC_BOLT_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>번개의 힘이 깃든 에너지 볼을 전방으로 발사한다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_BLIZARD_SKILL_NAME</t>
-  </si>
-  <si>
-    <t>블리자드</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_BLIZARD_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>하늘길을 열어 얼음 결정을 수엎이 쏟아붇는다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_DOUBLE_JUMP_SKILL_NAME</t>
-  </si>
-  <si>
-    <t>더블 점프</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_DOUBLE_JUMP_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>신성한 힘을 응축 시킨 후, 점프 후 공중에서 한 번 더 도약한다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_FLAME_SLASH_SKILL_NAME</t>
-  </si>
-  <si>
-    <t>플레임 슬래시</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_FLAME_SLASH_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>검날에 불꽃을 입혀 전방에 휘두른다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_MOON_BLADE_SKILL_NAME</t>
-  </si>
-  <si>
-    <t>문 블레이드</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_MOON_BLADE_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>달빛의 힘을 실은 검기를 전방으로 날린다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_SHADOW_PARTNER_SKILL_NAME</t>
-  </si>
-  <si>
-    <t>섀도우 파트너</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_SHADOW_PARTNER_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>어둠의 힘을 그림자에 깃들게한다.
+    <t xml:space="preserve">KEY_TEXT_SKILL_ARC_BOLT_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">아크볼트</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_ARC_BOLT_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">번개의 힘이 깃든 에너지 볼을 전방으로 발사한다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_BLIZARD_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">블리자드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_BLIZARD_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">하늘길을 열어 얼음 결정을 수엎이 쏟아붇는다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_DOUBLE_JUMP_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">더블 점프</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_DOUBLE_JUMP_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">신성한 힘을 응축 시킨 후, 점프 후 공중에서 한 번 더 도약한다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_FLAME_SLASH_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">플레임 슬래시</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_FLAME_SLASH_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">검날에 불꽃을 입혀 전방에 휘두른다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_MOON_BLADE_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">문 블레이드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_MOON_BLADE_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">달빛의 힘을 실은 검기를 전방으로 날린다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_SHADOW_PARTNER_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">섀도우 파트너</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_SHADOW_PARTNER_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">어둠의 힘을 그림자에 깃들게한다.
 나의 행동을 복제하는 그림자 분신을 생성한다.</t>
   </si>
   <si>
-    <t>KEY_TEXT_SKILL_WIND_DANCE_SKILL_NAME</t>
-  </si>
-  <si>
-    <t>윈드 댄스</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_SKILL_WIND_DANCE_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>바람 속에 녹아들어 시야에 들어온 모든 적들을 번갈아 가며 타격한다.</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_MONSTER_STAT_TABLE_DATA_NAME</t>
-  </si>
-  <si>
-    <t>거북 달팽이</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_MONSTER_STAT_TABLE_DATA_NAME_02</t>
-  </si>
-  <si>
-    <t>허니버블</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_MONSTER_STAT_TABLE_DATA_NAME_03</t>
-  </si>
-  <si>
-    <t>칵투스</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_MONSTER_STAT_TABLE_DATA_NAME_04</t>
-  </si>
-  <si>
-    <t>스네키</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0001_INTERACTION_DATA_NAME</t>
-  </si>
-  <si>
-    <t>그라함</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0001_INTERACTION_DATA_DIALOGUE_LINE_LIST_01</t>
-  </si>
-  <si>
-    <t>마을의 평화가 최우선일세</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0001_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_02</t>
-  </si>
-  <si>
-    <t>나도 왕년엔 이름 좀 날렸는데 말이야..</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0001_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_03</t>
-  </si>
-  <si>
-    <t>은퇴한 마법사지만, 지켜야할 주민들이 많아..</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0001_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_04</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0002_INTERACTION_DATA_NAME</t>
-  </si>
-  <si>
-    <t>드렉스</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0002_INTERACTION_DATA_DIALOGUE_LINE_LIST_01</t>
-  </si>
-  <si>
-    <t>달콤한 간식이 최고야</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0002_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_02</t>
-  </si>
-  <si>
-    <t>테토향이 좀 나나? 으하하</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0002_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_03</t>
-  </si>
-  <si>
-    <t>어디보자.. 이 주변에..</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0003_INTERACTION_DATA_NAME</t>
-  </si>
-  <si>
-    <t>알프레드</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0003_INTERACTION_DATA_DIALOGUE_LINE_LIST_01</t>
-  </si>
-  <si>
-    <t>없는 것 빼고 다 있답니다~?</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0003_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_02</t>
-  </si>
-  <si>
-    <t>거래는 언제든 환영이야~</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0003_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_03</t>
-  </si>
-  <si>
-    <t>내가 손에 든 건 안팔아!
+    <t xml:space="preserve">KEY_TEXT_SKILL_WIND_DANCE_SKILL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">윈드 댄스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_SKILL_WIND_DANCE_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바람 속에 녹아들어 시야에 들어온 모든 적들을 번갈아 가며 타격한다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_MONSTER_STAT_TABLE_DATA_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거북 달팽이</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_MONSTER_STAT_TABLE_DATA_NAME_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">허니버블</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_MONSTER_STAT_TABLE_DATA_NAME_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">칵투스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_MONSTER_STAT_TABLE_DATA_NAME_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">스네키</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0001_INTERACTION_DATA_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그라함</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0001_INTERACTION_DATA_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">마을의 평화가 최우선일세</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0001_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">나도 왕년엔 이름 좀 날렸는데 말이야..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0001_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">은퇴한 마법사지만, 지켜야할 주민들이 많아..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0001_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0002_INTERACTION_DATA_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">드렉스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0002_INTERACTION_DATA_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">달콤한 간식이 최고야</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0002_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">테토향이 좀 나나? 으하하</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0002_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">어디보자.. 이 주변에..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0003_INTERACTION_DATA_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">알프레드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0003_INTERACTION_DATA_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">없는 것 빼고 다 있답니다~?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0003_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거래는 언제든 환영이야~</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0003_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">내가 손에 든 건 안팔아!
 눈독들여도 소용 없어~</t>
   </si>
   <si>
-    <t>KEY_TEXT_NPC_0003_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_04</t>
-  </si>
-  <si>
-    <t>구매나 판매 뭐든 상관없어~
+    <t xml:space="preserve">KEY_TEXT_NPC_0003_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">구매나 판매 뭐든 상관없어~
 환영하네!</t>
   </si>
   <si>
-    <t>KEY_TEXT_NPC_0004_INTERACTION_DATA_NAME</t>
-  </si>
-  <si>
-    <t>앤트리</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0004_INTERACTION_DATA_DIALOGUE_LINE_LIST_01</t>
-  </si>
-  <si>
-    <t>꾸이이잉..</t>
-  </si>
-  <si>
-    <t>KEY_TEXT_NPC_0004_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_02</t>
-  </si>
-  <si>
-    <t>꾸잉..</t>
+    <t xml:space="preserve">KEY_TEXT_NPC_0004_INTERACTION_DATA_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">앤트리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0004_INTERACTION_DATA_DIALOGUE_LINE_LIST_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">꾸이이잉..</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_NPC_0004_INTERACTION_DATA_DIALOGUE_LINE_LIST_01_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">꾸잉..</t>
   </si>
   <si>
     <r>
@@ -604,7 +598,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>내가</t>
+      <t xml:space="preserve">내가</t>
     </r>
     <r>
       <rPr>
@@ -621,7 +615,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>년만</t>
+      <t xml:space="preserve">년만</t>
     </r>
     <r>
       <rPr>
@@ -638,7 +632,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>젊었어도</t>
+      <t xml:space="preserve">젊었어도</t>
     </r>
     <r>
       <rPr>
@@ -655,7 +649,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>으이</t>
+      <t xml:space="preserve">으이</t>
     </r>
     <r>
       <rPr>
@@ -673,7 +667,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>자네도</t>
+      <t xml:space="preserve">자네도</t>
     </r>
     <r>
       <rPr>
@@ -690,7 +684,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>이라고</t>
+      <t xml:space="preserve">이라고</t>
     </r>
     <r>
       <rPr>
@@ -707,7 +701,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>들어봤을테지</t>
+      <t xml:space="preserve">들어봤을테지</t>
     </r>
     <r>
       <rPr>
@@ -715,7 +709,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>?</t>
+      <t xml:space="preserve">?</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -727,7 +721,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>달콤한</t>
+      <t xml:space="preserve">달콤한</t>
     </r>
     <r>
       <rPr>
@@ -744,7 +738,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>향이</t>
+      <t xml:space="preserve">향이</t>
     </r>
     <r>
       <rPr>
@@ -761,7 +755,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>나는</t>
+      <t xml:space="preserve">나는</t>
     </r>
     <r>
       <rPr>
@@ -778,7 +772,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>허니</t>
+      <t xml:space="preserve">허니</t>
     </r>
     <r>
       <rPr>
@@ -795,7 +789,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>젤리다</t>
+      <t xml:space="preserve">젤리다</t>
     </r>
     <r>
       <rPr>
@@ -803,7 +797,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>.</t>
+      <t xml:space="preserve">.</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -815,7 +809,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>초보자의 브론즈</t>
+      <t xml:space="preserve">초보자의 브론즈</t>
     </r>
     <r>
       <rPr>
@@ -832,15 +826,46 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>소드</t>
+      <t xml:space="preserve">소드</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_CONTENT_DOWNLOAD_IN_PROGRESS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">업데이트 파일을 다운로드하고 있습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_CONTENT_DOWNLOAD_VERIFYING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">다운로드한 콘텐츠를 확인하고 있습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_CONTENT_DOWNLOAD_VERIFYING_STATUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">콘텐츠 확인 중...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_CONTENT_DOWNLOAD_COMPLETED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">업데이트 파일 다운로드가 완료됐습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_CONTENT_DOWNLOAD_COMPLETED_STATUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">다운로드 완료</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="6">
     <font>
       <sz val="11"/>
@@ -915,11 +940,11 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1136,6 +1161,7 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
@@ -1143,6 +1169,7 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
@@ -1150,6 +1177,7 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
           <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
@@ -1213,7 +1241,7 @@
   <a:objectDefaults>
     <a:lnDef>
       <a:spPr/>
-      <a:bodyPr/>
+      <a:bodyPr rtlCol="0"/>
       <a:lstStyle/>
       <a:style>
         <a:lnRef idx="2">
@@ -1241,8 +1269,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C93"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="3" width="36" customWidth="1"/>
@@ -1292,982 +1320,1037 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>185</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>186</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>187</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>188</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>189</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>190</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>191</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>192</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>193</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>194</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="16.5">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>184</v>
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="16.5">
       <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
+        <v>29</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>184</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C21" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C22" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="B23" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C23" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C24" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C26" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="B27" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B28" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="16.5">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>57</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>183</v>
+        <v>47</v>
+      </c>
+      <c r="B30" t="s">
+        <v>48</v>
       </c>
       <c r="C30" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B31" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C31" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B32" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C32" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="B33" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="C33" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="C34" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="16.5">
       <c r="A35" t="s">
-        <v>66</v>
-      </c>
-      <c r="B35" t="s">
-        <v>67</v>
+        <v>57</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>183</v>
       </c>
       <c r="C35" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B38" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="B39" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="C39" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B40" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C40" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B41" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C41" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B42" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C42" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="B43" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C43" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B44" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C44" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B45" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="C45" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B46" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C46" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="B47" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C47" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="B48" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C48" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="B49" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="C49" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B50" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="C50" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="B51" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="C51" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="B52" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="C52" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B53" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="C53" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B54" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C54" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B55" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C55" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B56" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C56" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="B57" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C57" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B58" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C58" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B59" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C59" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B60" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C60" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B61" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C61" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="B62" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C62" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="B63" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C63" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="B64" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C64" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="B65" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C65" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="B66" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C66" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B67" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C67" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="B68" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="C68" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="B69" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C69" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="B70" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="C70" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="B71" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="C71" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B72" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C72" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="B73" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C73" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B74" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C74" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="B75" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C75" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="B76" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C76" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="B77" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C77" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="B78" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="C78" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="B79" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="C79" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="B80" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C80" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" ht="14.25" customHeight="1">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>157</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>182</v>
+        <v>147</v>
+      </c>
+      <c r="B81" t="s">
+        <v>148</v>
       </c>
       <c r="C81" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="B82" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="C82" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="B83" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="C83" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="B84" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="C84" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="B85" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="C85" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" ht="14.25" customHeight="1">
       <c r="A86" t="s">
-        <v>166</v>
-      </c>
-      <c r="B86" t="s">
-        <v>167</v>
+        <v>157</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>182</v>
       </c>
       <c r="C86" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="B87" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C87" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="B88" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="C88" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="B89" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="C89" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="B90" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C90" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="B91" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="C91" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="B92" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="C92" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
+        <v>170</v>
+      </c>
+      <c r="B93" t="s">
+        <v>171</v>
+      </c>
+      <c r="C93" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" t="s">
+        <v>172</v>
+      </c>
+      <c r="B94" t="s">
+        <v>173</v>
+      </c>
+      <c r="C94" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3">
+      <c r="A95" t="s">
+        <v>174</v>
+      </c>
+      <c r="B95" t="s">
+        <v>175</v>
+      </c>
+      <c r="C95" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3">
+      <c r="A96" t="s">
+        <v>176</v>
+      </c>
+      <c r="B96" t="s">
+        <v>177</v>
+      </c>
+      <c r="C96" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" t="s">
+        <v>178</v>
+      </c>
+      <c r="B97" t="s">
+        <v>179</v>
+      </c>
+      <c r="C97" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" t="s">
         <v>180</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B98" t="s">
         <v>181</v>
       </c>
-      <c r="C93" t="s">
+      <c r="C98" t="s">
         <v>180</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[ UI ] Change content download rejection to exit
</commit_message>
<xml_diff>
--- a/Assets/RawData/Excel/Text/TextTableData.xlsx
+++ b/Assets/RawData/Excel/Text/TextTableData.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="198">
   <si>
     <t xml:space="preserve">TextKey</t>
   </si>
@@ -859,6 +859,15 @@
   </si>
   <si>
     <t xml:space="preserve">다운로드 완료</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY_TEXT_UI_COMMON_EXIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">종료</t>
   </si>
 </sst>
 </file>
@@ -1270,7 +1279,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="3" width="36" customWidth="1"/>
@@ -2354,6 +2363,17 @@
         <v>180</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="s">
+        <v>196</v>
+      </c>
+      <c r="B99" t="s">
+        <v>197</v>
+      </c>
+      <c r="C99" t="s">
+        <v>196</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>